<commit_message>
Activity DashBoard Test case Upted
</commit_message>
<xml_diff>
--- a/Data/loginPage.xlsx
+++ b/Data/loginPage.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>userName</t>
   </si>
@@ -35,10 +35,22 @@
     <t>password</t>
   </si>
   <si>
+    <t>exportType</t>
+  </si>
+  <si>
     <t>tsL9urF6O/D/xURRxzj/8w==</t>
   </si>
   <si>
-    <t>tsL9urF6O/APwsPS+50KRA==</t>
+    <t>HeCM15nHKBI=</t>
+  </si>
+  <si>
+    <t>excel</t>
+  </si>
+  <si>
+    <t>vG9BolkT2AE=</t>
+  </si>
+  <si>
+    <t>pdf</t>
   </si>
 </sst>
 </file>
@@ -46,10 +58,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -980,31 +992,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="2" max="2" width="18.9047619047619" customWidth="1"/>
+    <col min="1" max="1" width="30.2857142857143" customWidth="1"/>
+    <col min="2" max="2" width="29.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="tsL9urF6O/APwsPS+50KRA=="/>
+    <hyperlink ref="B2" r:id="rId1" display="HeCM15nHKBI="/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>